<commit_message>
Complete problem 4 partition and resource analysis
</commit_message>
<xml_diff>
--- a/outputs/问题三运输与中继联合调度方案.xlsx
+++ b/outputs/问题三运输与中继联合调度方案.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="结果总览" sheetId="1" r:id="R00f69fea1710448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中继架次" sheetId="2" r:id="Re2a58027c5a94864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通信保障" sheetId="3" r:id="Rd85bfd2b7d5041fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联合时序" sheetId="4" r:id="R3374c39cbe7d4a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运输架次" sheetId="5" r:id="Ra873844c252a4cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐箱交付" sheetId="6" r:id="R333afcd28e214e33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="可行性检查" sheetId="7" r:id="R34d40d1c4667475c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_中继架次" sheetId="8" r:id="R7151121e5919429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_通信保障" sheetId="9" r:id="R4e5b9a6abbf54235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="结果总览" sheetId="1" r:id="Rcad092ef33854dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中继架次" sheetId="2" r:id="Rbcd6f86f0bb645d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通信保障" sheetId="3" r:id="R73e3809ae8e349cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联合时序" sheetId="4" r:id="R2401665f0b274fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运输架次" sheetId="5" r:id="R7a6f0cab7c8348ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐箱交付" sheetId="6" r:id="R04b64625045d4fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="可行性检查" sheetId="7" r:id="Rd5196906ff8144c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_中继架次" sheetId="8" r:id="R7a9a3327e24c4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_通信保障" sheetId="9" r:id="R92f69304f0a541a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1002,7 +1002,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>21个运输架次与4个中继架次协同执行。全部货箱零延误，运输全过程连续通信。</x:v>
+        <x:v>21个运输架次与4个中继架次协同执行。全部货箱零延误，通信抽样未发现中断。</x:v>
       </x:c>
       <x:c r="B4" s="5"/>
       <x:c r="C4" s="5"/>
@@ -1125,7 +1125,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="134" t="n">
-        <x:v>68.93074666524997</x:v>
+        <x:v>68.96540467147017</x:v>
       </x:c>
       <x:c r="B13" s="135"/>
       <x:c r="C13" s="136"/>
@@ -1135,7 +1135,7 @@
       <x:c r="F13" s="153"/>
       <x:c r="G13" s="154"/>
       <x:c r="I13" s="152" t="n">
-        <x:v>0.5787618840105667</x:v>
+        <x:v>0.5736196004616878</x:v>
       </x:c>
       <x:c r="J13" s="153"/>
       <x:c r="K13" s="154"/>
@@ -1230,19 +1230,19 @@
         <x:v>2861</x:v>
       </x:c>
       <x:c r="D19" s="162" t="n">
-        <x:v>6.300212852538834</x:v>
+        <x:v>3.6385703388850175</x:v>
       </x:c>
       <x:c r="E19" s="162" t="n">
-        <x:v>0.4853694474559518</x:v>
+        <x:v>1.1033172362430719</x:v>
       </x:c>
       <x:c r="F19" s="162" t="n">
-        <x:v>0.4853694474559518</x:v>
+        <x:v>1.1033172362430719</x:v>
       </x:c>
       <x:c r="H19" s="15" t="str">
         <x:v>中继能耗_kWh</x:v>
       </x:c>
       <x:c r="I19" s="24" t="n">
-        <x:v>4.303991958504183</x:v>
+        <x:v>4.3386499647243815</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1256,13 +1256,13 @@
         <x:v>2978</x:v>
       </x:c>
       <x:c r="D20" s="162" t="n">
-        <x:v>0.48130542457175807</x:v>
+        <x:v>0.966414710398368</x:v>
       </x:c>
       <x:c r="E20" s="162" t="n">
-        <x:v>18.677291136943282</x:v>
+        <x:v>18.661876794936575</x:v>
       </x:c>
       <x:c r="F20" s="162" t="n">
-        <x:v>0.48130542457175807</x:v>
+        <x:v>0.966414710398368</x:v>
       </x:c>
       <x:c r="H20" s="15" t="str">
         <x:v>运输完成_s</x:v>
@@ -1315,7 +1315,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="180" t="str">
-        <x:v>方案实现80箱零延误和全过程连续通信。为完成两架中继无人机的区域轮换，运输完成时间比问题二增加349.0秒；中继增加4.3040 kWh能耗，联合任务在8277.90秒结束。</x:v>
+        <x:v>方案实现80箱零延误，逐秒与切换边界加密抽样均未发现通信中断。为完成两架中继无人机的区域轮换，运输完成时间比问题二增加349.0秒；中继增加4.3386 kWh能耗，联合任务在8277.90秒结束。</x:v>
       </x:c>
       <x:c r="B24" s="181"/>
       <x:c r="C24" s="181"/>
@@ -1630,22 +1630,22 @@
         <x:v>3928.0643800924636</x:v>
       </x:c>
       <x:c r="O7" s="23" t="n">
-        <x:v>3098.3209829141283</x:v>
+        <x:v>3128.3209829141283</x:v>
       </x:c>
       <x:c r="P7" s="26" t="n">
         <x:v>0.1601091397969594</x:v>
       </x:c>
       <x:c r="Q7" s="26" t="n">
-        <x:v>0.9467091892237616</x:v>
+        <x:v>0.9558758558904282</x:v>
       </x:c>
       <x:c r="R7" s="26" t="n">
-        <x:v>1.106818329020721</x:v>
+        <x:v>1.1159849956873877</x:v>
       </x:c>
       <x:c r="S7" s="29" t="n">
-        <x:v>0.6541192721810247</x:v>
+        <x:v>0.6512546888476913</x:v>
       </x:c>
       <x:c r="T7" s="29" t="n">
-        <x:v>0.4541192721810247</x:v>
+        <x:v>0.4512546888476913</x:v>
       </x:c>
       <x:c r="U7" s="14" t="str">
         <x:v>Q2-01, Q2-02, Q2-09, Q2-11, Q2-12</x:v>
@@ -1665,19 +1665,19 @@
         <x:v>东部</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
-        <x:v>GRID-7-3-H300</x:v>
+        <x:v>GRID-7-2-H300</x:v>
       </x:c>
       <x:c r="F8" s="18" t="n">
         <x:v>109.2835966</x:v>
       </x:c>
       <x:c r="G8" s="18" t="n">
-        <x:v>23.0299769</x:v>
+        <x:v>23.0175933</x:v>
       </x:c>
       <x:c r="H8" s="21" t="n">
         <x:v>300</x:v>
       </x:c>
       <x:c r="I8" s="21" t="n">
-        <x:v>716.1956176757812</x:v>
+        <x:v>726.6973876953125</x:v>
       </x:c>
       <x:c r="J8" s="24" t="n">
         <x:v>0</x:v>
@@ -1686,31 +1686,31 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="L8" s="24" t="n">
-        <x:v>750.6049005426124</x:v>
+        <x:v>725.8760198745433</x:v>
       </x:c>
       <x:c r="M8" s="24" t="n">
         <x:v>2686</x:v>
       </x:c>
       <x:c r="N8" s="24" t="n">
-        <x:v>3275.646202015594</x:v>
+        <x:v>3251.792468849153</x:v>
       </x:c>
       <x:c r="O8" s="24" t="n">
-        <x:v>1935.3950994573875</x:v>
+        <x:v>1990.1239801254567</x:v>
       </x:c>
       <x:c r="P8" s="27" t="n">
-        <x:v>0.3037141348318586</x:v>
+        <x:v>0.287171480366272</x:v>
       </x:c>
       <x:c r="Q8" s="27" t="n">
-        <x:v>0.5913707248342017</x:v>
+        <x:v>0.6080934383716673</x:v>
       </x:c>
       <x:c r="R8" s="27" t="n">
-        <x:v>0.8950848596660603</x:v>
+        <x:v>0.8952649187379393</x:v>
       </x:c>
       <x:c r="S8" s="30" t="n">
-        <x:v>0.7202859813543562</x:v>
+        <x:v>0.720229712894394</x:v>
       </x:c>
       <x:c r="T8" s="30" t="n">
-        <x:v>0.5202859813543561</x:v>
+        <x:v>0.520229712894394</x:v>
       </x:c>
       <x:c r="U8" s="15" t="str">
         <x:v>Q2-05, Q2-06, Q2-07, Q2-08, Q2-13</x:v>
@@ -1730,19 +1730,19 @@
         <x:v>西部</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
-        <x:v>O01-S007-MID-H300</x:v>
+        <x:v>WEST-109.213585-23.021464-H300</x:v>
       </x:c>
       <x:c r="F9" s="18" t="n">
-        <x:v>109.2118354</x:v>
+        <x:v>109.2135854</x:v>
       </x:c>
       <x:c r="G9" s="18" t="n">
-        <x:v>23.01896405</x:v>
+        <x:v>23.02146405</x:v>
       </x:c>
       <x:c r="H9" s="21" t="n">
         <x:v>300</x:v>
       </x:c>
       <x:c r="I9" s="21" t="n">
-        <x:v>586.2146301269531</x:v>
+        <x:v>538.5837554931641</x:v>
       </x:c>
       <x:c r="J9" s="24" t="n">
         <x:v>4228.064380092464</x:v>
@@ -1751,31 +1751,31 @@
         <x:v>4408.064380092464</x:v>
       </x:c>
       <x:c r="L9" s="24" t="n">
-        <x:v>4703.824952219404</x:v>
+        <x:v>4692.774413082056</x:v>
       </x:c>
       <x:c r="M9" s="24" t="n">
         <x:v>7377</x:v>
       </x:c>
       <x:c r="N9" s="24" t="n">
-        <x:v>7680.97012463752</x:v>
+        <x:v>7665.950345947355</x:v>
       </x:c>
       <x:c r="O9" s="24" t="n">
-        <x:v>2673.1750477805963</x:v>
+        <x:v>2714.2255869179444</x:v>
       </x:c>
       <x:c r="P9" s="27" t="n">
-        <x:v>0.13732331182936547</x:v>
+        <x:v>0.13363606466263872</x:v>
       </x:c>
       <x:c r="Q9" s="27" t="n">
-        <x:v>0.816803486821849</x:v>
+        <x:v>0.8293467071138164</x:v>
       </x:c>
       <x:c r="R9" s="27" t="n">
-        <x:v>0.9541267986512145</x:v>
+        <x:v>0.9629827717764552</x:v>
       </x:c>
       <x:c r="S9" s="30" t="n">
-        <x:v>0.7018353754214954</x:v>
+        <x:v>0.6990678838198578</x:v>
       </x:c>
       <x:c r="T9" s="30" t="n">
-        <x:v>0.5018353754214955</x:v>
+        <x:v>0.49906788381985784</x:v>
       </x:c>
       <x:c r="U9" s="15" t="str">
         <x:v>Q2-15, Q2-16, Q2-17, Q2-20</x:v>
@@ -1810,13 +1810,13 @@
         <x:v>539.3646392822266</x:v>
       </x:c>
       <x:c r="J10" s="25" t="n">
-        <x:v>3575.646202015594</x:v>
+        <x:v>3551.792468849153</x:v>
       </x:c>
       <x:c r="K10" s="25" t="n">
-        <x:v>3755.646202015594</x:v>
+        <x:v>3731.792468849153</x:v>
       </x:c>
       <x:c r="L10" s="25" t="n">
-        <x:v>4324.243056881041</x:v>
+        <x:v>4300.3893237146</x:v>
       </x:c>
       <x:c r="M10" s="25" t="n">
         <x:v>7705</x:v>
@@ -1825,22 +1825,22 @@
         <x:v>8277.9022414723</x:v>
       </x:c>
       <x:c r="O10" s="25" t="n">
-        <x:v>3380.7569431189586</x:v>
+        <x:v>3434.6106762853997</x:v>
       </x:c>
       <x:c r="P10" s="28" t="n">
         <x:v>0.3149529052131712</x:v>
       </x:c>
       <x:c r="Q10" s="28" t="n">
-        <x:v>1.0330090659530153</x:v>
+        <x:v>1.0494643733094278</x:v>
       </x:c>
       <x:c r="R10" s="28" t="n">
-        <x:v>1.3479619711661865</x:v>
+        <x:v>1.364417278522599</x:v>
       </x:c>
       <x:c r="S10" s="31" t="n">
-        <x:v>0.5787618840105667</x:v>
+        <x:v>0.5736196004616878</x:v>
       </x:c>
       <x:c r="T10" s="31" t="n">
-        <x:v>0.3787618840105667</x:v>
+        <x:v>0.3736196004616878</x:v>
       </x:c>
       <x:c r="U10" s="16" t="str">
         <x:v>Q2-14, Q2-18, Q2-19</x:v>
@@ -1893,7 +1893,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>直连不可用时切换为空中中继；最终按1秒采样验证，通信中断样本为0。</x:v>
+        <x:v>直连不可用时切换为空中中继；逐秒采样和切换边界加密检查均未发现通信中断。</x:v>
       </x:c>
       <x:c r="B4" s="5"/>
       <x:c r="C4" s="5"/>
@@ -1936,10 +1936,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
         <x:v>G01直连</x:v>
@@ -1954,13 +1954,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C8" s="33" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="D8" s="33" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="E8" s="33" t="n">
-        <x:v>856</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="F8" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -1977,13 +1977,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C9" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="D9" s="24" t="n">
         <x:v>2007.8</x:v>
       </x:c>
       <x:c r="E9" s="24" t="n">
-        <x:v>401.79999999999995</x:v>
+        <x:v>400.79999999999995</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2001,10 +2001,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="E10" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2019,13 +2019,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C11" s="33" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="D11" s="33" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="E11" s="33" t="n">
-        <x:v>856</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="F11" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2042,13 +2042,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C12" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="D12" s="24" t="n">
         <x:v>2007.8</x:v>
       </x:c>
       <x:c r="E12" s="24" t="n">
-        <x:v>401.79999999999995</x:v>
+        <x:v>400.79999999999995</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2108,10 +2108,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D15" s="24" t="n">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="E15" s="24" t="n">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="F15" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2126,13 +2126,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C16" s="33" t="n">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D16" s="33" t="n">
-        <x:v>1554</x:v>
+        <x:v>1555</x:v>
       </x:c>
       <x:c r="E16" s="33" t="n">
-        <x:v>798</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="F16" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2149,13 +2149,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C17" s="24" t="n">
-        <x:v>1554</x:v>
+        <x:v>1555</x:v>
       </x:c>
       <x:c r="D17" s="24" t="n">
         <x:v>1930.9</x:v>
       </x:c>
       <x:c r="E17" s="24" t="n">
-        <x:v>376.9000000000001</x:v>
+        <x:v>375.9000000000001</x:v>
       </x:c>
       <x:c r="F17" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2173,10 +2173,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D18" s="24" t="n">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="E18" s="24" t="n">
-        <x:v>744</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="F18" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2191,13 +2191,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C19" s="33" t="n">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="D19" s="33" t="n">
-        <x:v>1146</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="E19" s="33" t="n">
-        <x:v>395</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="F19" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2214,13 +2214,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C20" s="24" t="n">
-        <x:v>1146</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="D20" s="24" t="n">
         <x:v>1517.5</x:v>
       </x:c>
       <x:c r="E20" s="24" t="n">
-        <x:v>371.5</x:v>
+        <x:v>370.5</x:v>
       </x:c>
       <x:c r="F20" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2238,10 +2238,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D21" s="24" t="n">
-        <x:v>850</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="E21" s="24" t="n">
-        <x:v>843</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="F21" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2256,13 +2256,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C22" s="33" t="n">
-        <x:v>850</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="D22" s="33" t="n">
-        <x:v>1483</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="E22" s="33" t="n">
-        <x:v>633</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="F22" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2279,13 +2279,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C23" s="24" t="n">
-        <x:v>1483</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="D23" s="24" t="n">
         <x:v>1996</x:v>
       </x:c>
       <x:c r="E23" s="24" t="n">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F23" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2303,10 +2303,10 @@
         <x:v>1517.5</x:v>
       </x:c>
       <x:c r="D24" s="24" t="n">
-        <x:v>2274</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="E24" s="24" t="n">
-        <x:v>756.5</x:v>
+        <x:v>755.5</x:v>
       </x:c>
       <x:c r="F24" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2321,13 +2321,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C25" s="33" t="n">
-        <x:v>2274</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="D25" s="33" t="n">
-        <x:v>2686</x:v>
+        <x:v>2687</x:v>
       </x:c>
       <x:c r="E25" s="33" t="n">
-        <x:v>412</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="F25" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2344,13 +2344,13 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C26" s="24" t="n">
-        <x:v>2686</x:v>
+        <x:v>2687</x:v>
       </x:c>
       <x:c r="D26" s="24" t="n">
         <x:v>3072.1</x:v>
       </x:c>
       <x:c r="E26" s="24" t="n">
-        <x:v>386.0999999999999</x:v>
+        <x:v>385.0999999999999</x:v>
       </x:c>
       <x:c r="F26" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2368,10 +2368,10 @@
         <x:v>1560.9</x:v>
       </x:c>
       <x:c r="D27" s="24" t="n">
-        <x:v>2430</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="E27" s="24" t="n">
-        <x:v>869.0999999999999</x:v>
+        <x:v>868.0999999999999</x:v>
       </x:c>
       <x:c r="F27" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2386,13 +2386,13 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C28" s="33" t="n">
-        <x:v>2430</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="D28" s="33" t="n">
-        <x:v>2431</x:v>
+        <x:v>2432</x:v>
       </x:c>
       <x:c r="E28" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F28" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2402,25 +2402,27 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="15" t="str">
+      <x:c r="A29" s="32" t="str">
         <x:v>Q2-09</x:v>
       </x:c>
-      <x:c r="B29" s="15" t="str">
+      <x:c r="B29" s="32" t="str">
         <x:v>阶段3</x:v>
       </x:c>
-      <x:c r="C29" s="24" t="n">
-        <x:v>2431</x:v>
-      </x:c>
-      <x:c r="D29" s="24" t="n">
-        <x:v>2433</x:v>
-      </x:c>
-      <x:c r="E29" s="24" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F29" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G29" s="15"/>
+      <x:c r="C29" s="33" t="n">
+        <x:v>2432</x:v>
+      </x:c>
+      <x:c r="D29" s="33" t="n">
+        <x:v>3010</x:v>
+      </x:c>
+      <x:c r="E29" s="33" t="n">
+        <x:v>578</x:v>
+      </x:c>
+      <x:c r="F29" s="32" t="str">
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="G29" s="32" t="str">
+        <x:v>R-M01</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="str">
@@ -2430,13 +2432,13 @@
         <x:v>阶段4</x:v>
       </x:c>
       <x:c r="C30" s="33" t="n">
-        <x:v>2433</x:v>
+        <x:v>3010</x:v>
       </x:c>
       <x:c r="D30" s="33" t="n">
-        <x:v>3009</x:v>
+        <x:v>3013</x:v>
       </x:c>
       <x:c r="E30" s="33" t="n">
-        <x:v>576</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F30" s="32" t="str">
         <x:v>空中中继</x:v>
@@ -2453,13 +2455,13 @@
         <x:v>阶段5</x:v>
       </x:c>
       <x:c r="C31" s="24" t="n">
-        <x:v>3009</x:v>
+        <x:v>3013</x:v>
       </x:c>
       <x:c r="D31" s="24" t="n">
-        <x:v>3011</x:v>
+        <x:v>3468.4</x:v>
       </x:c>
       <x:c r="E31" s="24" t="n">
-        <x:v>2</x:v>
+        <x:v>455.4000000000001</x:v>
       </x:c>
       <x:c r="F31" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2467,43 +2469,41 @@
       <x:c r="G31" s="15"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="32" t="str">
-        <x:v>Q2-09</x:v>
-      </x:c>
-      <x:c r="B32" s="32" t="str">
-        <x:v>阶段6</x:v>
-      </x:c>
-      <x:c r="C32" s="33" t="n">
-        <x:v>3011</x:v>
-      </x:c>
-      <x:c r="D32" s="33" t="n">
-        <x:v>3012</x:v>
-      </x:c>
-      <x:c r="E32" s="33" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F32" s="32" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="G32" s="32" t="str">
-        <x:v>R-M01</x:v>
-      </x:c>
+      <x:c r="A32" s="15" t="str">
+        <x:v>Q2-10</x:v>
+      </x:c>
+      <x:c r="B32" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C32" s="24" t="n">
+        <x:v>1693.5</x:v>
+      </x:c>
+      <x:c r="D32" s="24" t="n">
+        <x:v>3189</x:v>
+      </x:c>
+      <x:c r="E32" s="24" t="n">
+        <x:v>1495.5</x:v>
+      </x:c>
+      <x:c r="F32" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G32" s="15"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="15" t="str">
-        <x:v>Q2-09</x:v>
+        <x:v>Q2-11</x:v>
       </x:c>
       <x:c r="B33" s="15" t="str">
-        <x:v>阶段7</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C33" s="24" t="n">
-        <x:v>3012</x:v>
+        <x:v>1930.9</x:v>
       </x:c>
       <x:c r="D33" s="24" t="n">
-        <x:v>3468.4</x:v>
+        <x:v>2614</x:v>
       </x:c>
       <x:c r="E33" s="24" t="n">
-        <x:v>456.4000000000001</x:v>
+        <x:v>683.0999999999999</x:v>
       </x:c>
       <x:c r="F33" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2511,41 +2511,43 @@
       <x:c r="G33" s="15"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="15" t="str">
-        <x:v>Q2-10</x:v>
-      </x:c>
-      <x:c r="B34" s="15" t="str">
-        <x:v>阶段1</x:v>
-      </x:c>
-      <x:c r="C34" s="24" t="n">
-        <x:v>1693.5</x:v>
-      </x:c>
-      <x:c r="D34" s="24" t="n">
-        <x:v>3189</x:v>
-      </x:c>
-      <x:c r="E34" s="24" t="n">
-        <x:v>1495.5</x:v>
-      </x:c>
-      <x:c r="F34" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G34" s="15"/>
+      <x:c r="A34" s="32" t="str">
+        <x:v>Q2-11</x:v>
+      </x:c>
+      <x:c r="B34" s="32" t="str">
+        <x:v>阶段2</x:v>
+      </x:c>
+      <x:c r="C34" s="33" t="n">
+        <x:v>2614</x:v>
+      </x:c>
+      <x:c r="D34" s="33" t="n">
+        <x:v>3356</x:v>
+      </x:c>
+      <x:c r="E34" s="33" t="n">
+        <x:v>742</x:v>
+      </x:c>
+      <x:c r="F34" s="32" t="str">
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="G34" s="32" t="str">
+        <x:v>R-M01</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="15" t="str">
         <x:v>Q2-11</x:v>
       </x:c>
       <x:c r="B35" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C35" s="24" t="n">
-        <x:v>1930.9</x:v>
+        <x:v>3356</x:v>
       </x:c>
       <x:c r="D35" s="24" t="n">
-        <x:v>2615</x:v>
+        <x:v>3690.8</x:v>
       </x:c>
       <x:c r="E35" s="24" t="n">
-        <x:v>684.0999999999999</x:v>
+        <x:v>334.8000000000002</x:v>
       </x:c>
       <x:c r="F35" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2553,64 +2555,64 @@
       <x:c r="G35" s="15"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="32" t="str">
-        <x:v>Q2-11</x:v>
-      </x:c>
-      <x:c r="B36" s="32" t="str">
+      <x:c r="A36" s="15" t="str">
+        <x:v>Q2-12</x:v>
+      </x:c>
+      <x:c r="B36" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C36" s="24" t="n">
+        <x:v>1996</x:v>
+      </x:c>
+      <x:c r="D36" s="24" t="n">
+        <x:v>2745</x:v>
+      </x:c>
+      <x:c r="E36" s="24" t="n">
+        <x:v>749</x:v>
+      </x:c>
+      <x:c r="F36" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G36" s="15"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="32" t="str">
+        <x:v>Q2-12</x:v>
+      </x:c>
+      <x:c r="B37" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C36" s="33" t="n">
-        <x:v>2615</x:v>
-      </x:c>
-      <x:c r="D36" s="33" t="n">
-        <x:v>3355</x:v>
-      </x:c>
-      <x:c r="E36" s="33" t="n">
-        <x:v>740</x:v>
-      </x:c>
-      <x:c r="F36" s="32" t="str">
+      <x:c r="C37" s="33" t="n">
+        <x:v>2745</x:v>
+      </x:c>
+      <x:c r="D37" s="33" t="n">
+        <x:v>3603</x:v>
+      </x:c>
+      <x:c r="E37" s="33" t="n">
+        <x:v>858</x:v>
+      </x:c>
+      <x:c r="F37" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G36" s="32" t="str">
+      <x:c r="G37" s="32" t="str">
         <x:v>R-M01</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="15" t="str">
-        <x:v>Q2-11</x:v>
-      </x:c>
-      <x:c r="B37" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C37" s="24" t="n">
-        <x:v>3355</x:v>
-      </x:c>
-      <x:c r="D37" s="24" t="n">
-        <x:v>3690.8</x:v>
-      </x:c>
-      <x:c r="E37" s="24" t="n">
-        <x:v>335.8000000000002</x:v>
-      </x:c>
-      <x:c r="F37" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G37" s="15"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="15" t="str">
         <x:v>Q2-12</x:v>
       </x:c>
       <x:c r="B38" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C38" s="24" t="n">
-        <x:v>1996</x:v>
+        <x:v>3603</x:v>
       </x:c>
       <x:c r="D38" s="24" t="n">
-        <x:v>2746</x:v>
+        <x:v>4003.8</x:v>
       </x:c>
       <x:c r="E38" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>400.8000000000002</x:v>
       </x:c>
       <x:c r="F38" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2618,64 +2620,64 @@
       <x:c r="G38" s="15"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="32" t="str">
-        <x:v>Q2-12</x:v>
-      </x:c>
-      <x:c r="B39" s="32" t="str">
+      <x:c r="A39" s="15" t="str">
+        <x:v>Q2-13</x:v>
+      </x:c>
+      <x:c r="B39" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C39" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="24" t="n">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="E39" s="24" t="n">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="F39" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G39" s="15"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="32" t="str">
+        <x:v>Q2-13</x:v>
+      </x:c>
+      <x:c r="B40" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C39" s="33" t="n">
-        <x:v>2746</x:v>
-      </x:c>
-      <x:c r="D39" s="33" t="n">
-        <x:v>3602</x:v>
-      </x:c>
-      <x:c r="E39" s="33" t="n">
-        <x:v>856</x:v>
-      </x:c>
-      <x:c r="F39" s="32" t="str">
+      <x:c r="C40" s="33" t="n">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="D40" s="33" t="n">
+        <x:v>1417</x:v>
+      </x:c>
+      <x:c r="E40" s="33" t="n">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="F40" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G39" s="32" t="str">
-        <x:v>R-M01</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="15" t="str">
-        <x:v>Q2-12</x:v>
-      </x:c>
-      <x:c r="B40" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C40" s="24" t="n">
-        <x:v>3602</x:v>
-      </x:c>
-      <x:c r="D40" s="24" t="n">
-        <x:v>4003.8</x:v>
-      </x:c>
-      <x:c r="E40" s="24" t="n">
-        <x:v>401.8000000000002</x:v>
-      </x:c>
-      <x:c r="F40" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G40" s="15"/>
+      <x:c r="G40" s="32" t="str">
+        <x:v>R-M02</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="15" t="str">
         <x:v>Q2-13</x:v>
       </x:c>
       <x:c r="B41" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C41" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="D41" s="24" t="n">
-        <x:v>813</x:v>
+        <x:v>1928.9623510146916</x:v>
       </x:c>
       <x:c r="E41" s="24" t="n">
-        <x:v>813</x:v>
+        <x:v>511.96235101469165</x:v>
       </x:c>
       <x:c r="F41" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2683,64 +2685,64 @@
       <x:c r="G41" s="15"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="32" t="str">
-        <x:v>Q2-13</x:v>
-      </x:c>
-      <x:c r="B42" s="32" t="str">
+      <x:c r="A42" s="15" t="str">
+        <x:v>Q2-14</x:v>
+      </x:c>
+      <x:c r="B42" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C42" s="24" t="n">
+        <x:v>3362</x:v>
+      </x:c>
+      <x:c r="D42" s="24" t="n">
+        <x:v>4324</x:v>
+      </x:c>
+      <x:c r="E42" s="24" t="n">
+        <x:v>962</x:v>
+      </x:c>
+      <x:c r="F42" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G42" s="15"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="32" t="str">
+        <x:v>Q2-14</x:v>
+      </x:c>
+      <x:c r="B43" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C42" s="33" t="n">
-        <x:v>813</x:v>
-      </x:c>
-      <x:c r="D42" s="33" t="n">
-        <x:v>1416</x:v>
-      </x:c>
-      <x:c r="E42" s="33" t="n">
-        <x:v>603</x:v>
-      </x:c>
-      <x:c r="F42" s="32" t="str">
+      <x:c r="C43" s="33" t="n">
+        <x:v>4324</x:v>
+      </x:c>
+      <x:c r="D43" s="33" t="n">
+        <x:v>5159</x:v>
+      </x:c>
+      <x:c r="E43" s="33" t="n">
+        <x:v>835</x:v>
+      </x:c>
+      <x:c r="F43" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G42" s="32" t="str">
-        <x:v>R-M02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="15" t="str">
-        <x:v>Q2-13</x:v>
-      </x:c>
-      <x:c r="B43" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C43" s="24" t="n">
-        <x:v>1416</x:v>
-      </x:c>
-      <x:c r="D43" s="24" t="n">
-        <x:v>1928.9623510146916</x:v>
-      </x:c>
-      <x:c r="E43" s="24" t="n">
-        <x:v>512.9623510146916</x:v>
-      </x:c>
-      <x:c r="F43" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G43" s="15"/>
+      <x:c r="G43" s="32" t="str">
+        <x:v>R-M04</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="15" t="str">
         <x:v>Q2-14</x:v>
       </x:c>
       <x:c r="B44" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C44" s="24" t="n">
-        <x:v>3362</x:v>
+        <x:v>5159</x:v>
       </x:c>
       <x:c r="D44" s="24" t="n">
-        <x:v>4325</x:v>
+        <x:v>5667.2</x:v>
       </x:c>
       <x:c r="E44" s="24" t="n">
-        <x:v>963</x:v>
+        <x:v>508.1999999999998</x:v>
       </x:c>
       <x:c r="F44" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2748,64 +2750,64 @@
       <x:c r="G44" s="15"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="32" t="str">
-        <x:v>Q2-14</x:v>
-      </x:c>
-      <x:c r="B45" s="32" t="str">
+      <x:c r="A45" s="15" t="str">
+        <x:v>Q2-15</x:v>
+      </x:c>
+      <x:c r="B45" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C45" s="24" t="n">
+        <x:v>3817.4</x:v>
+      </x:c>
+      <x:c r="D45" s="24" t="n">
+        <x:v>4703</x:v>
+      </x:c>
+      <x:c r="E45" s="24" t="n">
+        <x:v>885.5999999999999</x:v>
+      </x:c>
+      <x:c r="F45" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G45" s="15"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="32" t="str">
+        <x:v>Q2-15</x:v>
+      </x:c>
+      <x:c r="B46" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C45" s="33" t="n">
-        <x:v>4325</x:v>
-      </x:c>
-      <x:c r="D45" s="33" t="n">
-        <x:v>5158</x:v>
-      </x:c>
-      <x:c r="E45" s="33" t="n">
-        <x:v>833</x:v>
-      </x:c>
-      <x:c r="F45" s="32" t="str">
+      <x:c r="C46" s="33" t="n">
+        <x:v>4703</x:v>
+      </x:c>
+      <x:c r="D46" s="33" t="n">
+        <x:v>5709</x:v>
+      </x:c>
+      <x:c r="E46" s="33" t="n">
+        <x:v>1006</x:v>
+      </x:c>
+      <x:c r="F46" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G45" s="32" t="str">
-        <x:v>R-M04</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="15" t="str">
-        <x:v>Q2-14</x:v>
-      </x:c>
-      <x:c r="B46" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C46" s="24" t="n">
-        <x:v>5158</x:v>
-      </x:c>
-      <x:c r="D46" s="24" t="n">
-        <x:v>5667.2</x:v>
-      </x:c>
-      <x:c r="E46" s="24" t="n">
-        <x:v>509.1999999999998</x:v>
-      </x:c>
-      <x:c r="F46" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G46" s="15"/>
+      <x:c r="G46" s="32" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="15" t="str">
         <x:v>Q2-15</x:v>
       </x:c>
       <x:c r="B47" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C47" s="24" t="n">
-        <x:v>3817.4</x:v>
+        <x:v>5709</x:v>
       </x:c>
       <x:c r="D47" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>6187.3</x:v>
       </x:c>
       <x:c r="E47" s="24" t="n">
-        <x:v>886.5999999999999</x:v>
+        <x:v>478.3000000000002</x:v>
       </x:c>
       <x:c r="F47" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2813,64 +2815,64 @@
       <x:c r="G47" s="15"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="32" t="str">
-        <x:v>Q2-15</x:v>
-      </x:c>
-      <x:c r="B48" s="32" t="str">
+      <x:c r="A48" s="15" t="str">
+        <x:v>Q2-16</x:v>
+      </x:c>
+      <x:c r="B48" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C48" s="24" t="n">
+        <x:v>3906.5</x:v>
+      </x:c>
+      <x:c r="D48" s="24" t="n">
+        <x:v>4703</x:v>
+      </x:c>
+      <x:c r="E48" s="24" t="n">
+        <x:v>796.5</x:v>
+      </x:c>
+      <x:c r="F48" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G48" s="15"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="32" t="str">
+        <x:v>Q2-16</x:v>
+      </x:c>
+      <x:c r="B49" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C48" s="33" t="n">
-        <x:v>4704</x:v>
-      </x:c>
-      <x:c r="D48" s="33" t="n">
-        <x:v>5708</x:v>
-      </x:c>
-      <x:c r="E48" s="33" t="n">
-        <x:v>1004</x:v>
-      </x:c>
-      <x:c r="F48" s="32" t="str">
+      <x:c r="C49" s="33" t="n">
+        <x:v>4703</x:v>
+      </x:c>
+      <x:c r="D49" s="33" t="n">
+        <x:v>5552</x:v>
+      </x:c>
+      <x:c r="E49" s="33" t="n">
+        <x:v>849</x:v>
+      </x:c>
+      <x:c r="F49" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G48" s="32" t="str">
+      <x:c r="G49" s="32" t="str">
         <x:v>R-M03</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="15" t="str">
-        <x:v>Q2-15</x:v>
-      </x:c>
-      <x:c r="B49" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C49" s="24" t="n">
-        <x:v>5708</x:v>
-      </x:c>
-      <x:c r="D49" s="24" t="n">
-        <x:v>6187.3</x:v>
-      </x:c>
-      <x:c r="E49" s="24" t="n">
-        <x:v>479.3000000000002</x:v>
-      </x:c>
-      <x:c r="F49" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G49" s="15"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="15" t="str">
         <x:v>Q2-16</x:v>
       </x:c>
       <x:c r="B50" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C50" s="24" t="n">
-        <x:v>3906.5</x:v>
+        <x:v>5552</x:v>
       </x:c>
       <x:c r="D50" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>5986.8</x:v>
       </x:c>
       <x:c r="E50" s="24" t="n">
-        <x:v>797.5</x:v>
+        <x:v>434.8000000000002</x:v>
       </x:c>
       <x:c r="F50" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2878,64 +2880,64 @@
       <x:c r="G50" s="15"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="32" t="str">
-        <x:v>Q2-16</x:v>
-      </x:c>
-      <x:c r="B51" s="32" t="str">
+      <x:c r="A51" s="15" t="str">
+        <x:v>Q2-17</x:v>
+      </x:c>
+      <x:c r="B51" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C51" s="24" t="n">
+        <x:v>4813.7</x:v>
+      </x:c>
+      <x:c r="D51" s="24" t="n">
+        <x:v>5522</x:v>
+      </x:c>
+      <x:c r="E51" s="24" t="n">
+        <x:v>708.3000000000002</x:v>
+      </x:c>
+      <x:c r="F51" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G51" s="15"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="32" t="str">
+        <x:v>Q2-17</x:v>
+      </x:c>
+      <x:c r="B52" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C51" s="33" t="n">
-        <x:v>4704</x:v>
-      </x:c>
-      <x:c r="D51" s="33" t="n">
-        <x:v>5551</x:v>
-      </x:c>
-      <x:c r="E51" s="33" t="n">
-        <x:v>847</x:v>
-      </x:c>
-      <x:c r="F51" s="32" t="str">
+      <x:c r="C52" s="33" t="n">
+        <x:v>5522</x:v>
+      </x:c>
+      <x:c r="D52" s="33" t="n">
+        <x:v>6046</x:v>
+      </x:c>
+      <x:c r="E52" s="33" t="n">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="F52" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G51" s="32" t="str">
+      <x:c r="G52" s="32" t="str">
         <x:v>R-M03</x:v>
       </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="15" t="str">
-        <x:v>Q2-16</x:v>
-      </x:c>
-      <x:c r="B52" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C52" s="24" t="n">
-        <x:v>5551</x:v>
-      </x:c>
-      <x:c r="D52" s="24" t="n">
-        <x:v>5986.8</x:v>
-      </x:c>
-      <x:c r="E52" s="24" t="n">
-        <x:v>435.8000000000002</x:v>
-      </x:c>
-      <x:c r="F52" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G52" s="15"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="15" t="str">
         <x:v>Q2-17</x:v>
       </x:c>
       <x:c r="B53" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C53" s="24" t="n">
-        <x:v>4813.7</x:v>
+        <x:v>6046</x:v>
       </x:c>
       <x:c r="D53" s="24" t="n">
-        <x:v>5523</x:v>
+        <x:v>6374.5</x:v>
       </x:c>
       <x:c r="E53" s="24" t="n">
-        <x:v>709.3000000000002</x:v>
+        <x:v>328.5</x:v>
       </x:c>
       <x:c r="F53" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -2943,64 +2945,64 @@
       <x:c r="G53" s="15"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="32" t="str">
-        <x:v>Q2-17</x:v>
-      </x:c>
-      <x:c r="B54" s="32" t="str">
+      <x:c r="A54" s="15" t="str">
+        <x:v>Q2-18</x:v>
+      </x:c>
+      <x:c r="B54" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C54" s="24" t="n">
+        <x:v>5667.2</x:v>
+      </x:c>
+      <x:c r="D54" s="24" t="n">
+        <x:v>6508</x:v>
+      </x:c>
+      <x:c r="E54" s="24" t="n">
+        <x:v>840.8000000000002</x:v>
+      </x:c>
+      <x:c r="F54" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G54" s="15"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="32" t="str">
+        <x:v>Q2-18</x:v>
+      </x:c>
+      <x:c r="B55" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C54" s="33" t="n">
-        <x:v>5523</x:v>
-      </x:c>
-      <x:c r="D54" s="33" t="n">
-        <x:v>6045</x:v>
-      </x:c>
-      <x:c r="E54" s="33" t="n">
-        <x:v>522</x:v>
-      </x:c>
-      <x:c r="F54" s="32" t="str">
+      <x:c r="C55" s="33" t="n">
+        <x:v>6508</x:v>
+      </x:c>
+      <x:c r="D55" s="33" t="n">
+        <x:v>7457</x:v>
+      </x:c>
+      <x:c r="E55" s="33" t="n">
+        <x:v>949</x:v>
+      </x:c>
+      <x:c r="F55" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G54" s="32" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="15" t="str">
-        <x:v>Q2-17</x:v>
-      </x:c>
-      <x:c r="B55" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C55" s="24" t="n">
-        <x:v>6045</x:v>
-      </x:c>
-      <x:c r="D55" s="24" t="n">
-        <x:v>6374.5</x:v>
-      </x:c>
-      <x:c r="E55" s="24" t="n">
-        <x:v>329.5</x:v>
-      </x:c>
-      <x:c r="F55" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G55" s="15"/>
+      <x:c r="G55" s="32" t="str">
+        <x:v>R-M04</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="15" t="str">
         <x:v>Q2-18</x:v>
       </x:c>
       <x:c r="B56" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C56" s="24" t="n">
-        <x:v>5667.2</x:v>
+        <x:v>7457</x:v>
       </x:c>
       <x:c r="D56" s="24" t="n">
-        <x:v>6509</x:v>
+        <x:v>7871</x:v>
       </x:c>
       <x:c r="E56" s="24" t="n">
-        <x:v>841.8000000000002</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="F56" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -3008,64 +3010,64 @@
       <x:c r="G56" s="15"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="32" t="str">
-        <x:v>Q2-18</x:v>
-      </x:c>
-      <x:c r="B57" s="32" t="str">
+      <x:c r="A57" s="15" t="str">
+        <x:v>Q2-19</x:v>
+      </x:c>
+      <x:c r="B57" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C57" s="24" t="n">
+        <x:v>6187.3</x:v>
+      </x:c>
+      <x:c r="D57" s="24" t="n">
+        <x:v>7010</x:v>
+      </x:c>
+      <x:c r="E57" s="24" t="n">
+        <x:v>822.6999999999998</x:v>
+      </x:c>
+      <x:c r="F57" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G57" s="15"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="32" t="str">
+        <x:v>Q2-19</x:v>
+      </x:c>
+      <x:c r="B58" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C57" s="33" t="n">
-        <x:v>6509</x:v>
-      </x:c>
-      <x:c r="D57" s="33" t="n">
-        <x:v>7456</x:v>
-      </x:c>
-      <x:c r="E57" s="33" t="n">
-        <x:v>947</x:v>
-      </x:c>
-      <x:c r="F57" s="32" t="str">
+      <x:c r="C58" s="33" t="n">
+        <x:v>7010</x:v>
+      </x:c>
+      <x:c r="D58" s="33" t="n">
+        <x:v>7706</x:v>
+      </x:c>
+      <x:c r="E58" s="33" t="n">
+        <x:v>696</x:v>
+      </x:c>
+      <x:c r="F58" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G57" s="32" t="str">
+      <x:c r="G58" s="32" t="str">
         <x:v>R-M04</x:v>
       </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="15" t="str">
-        <x:v>Q2-18</x:v>
-      </x:c>
-      <x:c r="B58" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C58" s="24" t="n">
-        <x:v>7456</x:v>
-      </x:c>
-      <x:c r="D58" s="24" t="n">
-        <x:v>7871</x:v>
-      </x:c>
-      <x:c r="E58" s="24" t="n">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="F58" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G58" s="15"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="15" t="str">
         <x:v>Q2-19</x:v>
       </x:c>
       <x:c r="B59" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C59" s="24" t="n">
-        <x:v>6187.3</x:v>
+        <x:v>7706</x:v>
       </x:c>
       <x:c r="D59" s="24" t="n">
-        <x:v>7011</x:v>
+        <x:v>8067.4</x:v>
       </x:c>
       <x:c r="E59" s="24" t="n">
-        <x:v>823.6999999999998</x:v>
+        <x:v>361.39999999999964</x:v>
       </x:c>
       <x:c r="F59" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -3073,64 +3075,64 @@
       <x:c r="G59" s="15"/>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="32" t="str">
-        <x:v>Q2-19</x:v>
-      </x:c>
-      <x:c r="B60" s="32" t="str">
+      <x:c r="A60" s="15" t="str">
+        <x:v>Q2-20</x:v>
+      </x:c>
+      <x:c r="B60" s="15" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C60" s="24" t="n">
+        <x:v>5986.8</x:v>
+      </x:c>
+      <x:c r="D60" s="24" t="n">
+        <x:v>6787</x:v>
+      </x:c>
+      <x:c r="E60" s="24" t="n">
+        <x:v>800.1999999999998</x:v>
+      </x:c>
+      <x:c r="F60" s="15" t="str">
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="G60" s="15"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="32" t="str">
+        <x:v>Q2-20</x:v>
+      </x:c>
+      <x:c r="B61" s="32" t="str">
         <x:v>阶段2</x:v>
       </x:c>
-      <x:c r="C60" s="33" t="n">
-        <x:v>7011</x:v>
-      </x:c>
-      <x:c r="D60" s="33" t="n">
-        <x:v>7705</x:v>
-      </x:c>
-      <x:c r="E60" s="33" t="n">
-        <x:v>694</x:v>
-      </x:c>
-      <x:c r="F60" s="32" t="str">
+      <x:c r="C61" s="33" t="n">
+        <x:v>6787</x:v>
+      </x:c>
+      <x:c r="D61" s="33" t="n">
+        <x:v>7378</x:v>
+      </x:c>
+      <x:c r="E61" s="33" t="n">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="F61" s="32" t="str">
         <x:v>空中中继</x:v>
       </x:c>
-      <x:c r="G60" s="32" t="str">
-        <x:v>R-M04</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="15" t="str">
-        <x:v>Q2-19</x:v>
-      </x:c>
-      <x:c r="B61" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C61" s="24" t="n">
-        <x:v>7705</x:v>
-      </x:c>
-      <x:c r="D61" s="24" t="n">
-        <x:v>8067.4</x:v>
-      </x:c>
-      <x:c r="E61" s="24" t="n">
-        <x:v>362.39999999999964</x:v>
-      </x:c>
-      <x:c r="F61" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G61" s="15"/>
+      <x:c r="G61" s="32" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="15" t="str">
         <x:v>Q2-20</x:v>
       </x:c>
       <x:c r="B62" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C62" s="24" t="n">
-        <x:v>5986.8</x:v>
+        <x:v>7378</x:v>
       </x:c>
       <x:c r="D62" s="24" t="n">
-        <x:v>6788</x:v>
+        <x:v>7816.4</x:v>
       </x:c>
       <x:c r="E62" s="24" t="n">
-        <x:v>801.1999999999998</x:v>
+        <x:v>438.39999999999964</x:v>
       </x:c>
       <x:c r="F62" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -3138,69 +3140,25 @@
       <x:c r="G62" s="15"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="32" t="str">
-        <x:v>Q2-20</x:v>
-      </x:c>
-      <x:c r="B63" s="32" t="str">
-        <x:v>阶段2</x:v>
-      </x:c>
-      <x:c r="C63" s="33" t="n">
-        <x:v>6788</x:v>
-      </x:c>
-      <x:c r="D63" s="33" t="n">
-        <x:v>7377</x:v>
-      </x:c>
-      <x:c r="E63" s="33" t="n">
-        <x:v>589</x:v>
-      </x:c>
-      <x:c r="F63" s="32" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="G63" s="32" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="15" t="str">
-        <x:v>Q2-20</x:v>
-      </x:c>
-      <x:c r="B64" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C64" s="24" t="n">
-        <x:v>7377</x:v>
-      </x:c>
-      <x:c r="D64" s="24" t="n">
-        <x:v>7816.4</x:v>
-      </x:c>
-      <x:c r="E64" s="24" t="n">
-        <x:v>439.39999999999964</x:v>
-      </x:c>
-      <x:c r="F64" s="15" t="str">
+      <x:c r="A63" s="16" t="str">
+        <x:v>Q2-21</x:v>
+      </x:c>
+      <x:c r="B63" s="16" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C63" s="25" t="n">
+        <x:v>6374.5</x:v>
+      </x:c>
+      <x:c r="D63" s="25" t="n">
+        <x:v>7561.2</x:v>
+      </x:c>
+      <x:c r="E63" s="25" t="n">
+        <x:v>1186.6999999999998</x:v>
+      </x:c>
+      <x:c r="F63" s="16" t="str">
         <x:v>G01直连</x:v>
       </x:c>
-      <x:c r="G64" s="15"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="16" t="str">
-        <x:v>Q2-21</x:v>
-      </x:c>
-      <x:c r="B65" s="16" t="str">
-        <x:v>阶段1</x:v>
-      </x:c>
-      <x:c r="C65" s="25" t="n">
-        <x:v>6374.5</x:v>
-      </x:c>
-      <x:c r="D65" s="25" t="n">
-        <x:v>7561.2</x:v>
-      </x:c>
-      <x:c r="E65" s="25" t="n">
-        <x:v>1186.6999999999998</x:v>
-      </x:c>
-      <x:c r="F65" s="16" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="G65" s="16"/>
+      <x:c r="G63" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4245,7 +4203,7 @@
         <x:v>R-M04</x:v>
       </x:c>
       <x:c r="D31" s="48" t="n">
-        <x:v>3575.646202015594</x:v>
+        <x:v>3551.792468849153</x:v>
       </x:c>
       <x:c r="E31" s="49" t="str"/>
       <x:c r="F31" s="49" t="str"/>
@@ -8445,7 +8403,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="C14" s="38" t="str">
-        <x:v>最低 0.578762</x:v>
+        <x:v>最低 0.573620</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -8460,13 +8418,24 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="39" t="str">
+      <x:c r="A16" s="38" t="str">
+        <x:v>通信切换边界加密检查</x:v>
+      </x:c>
+      <x:c r="B16" s="38" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="C16" s="38" t="str">
+        <x:v>检查 1558 个边界样本，中断 0 点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="39" t="str">
         <x:v>连续通信</x:v>
       </x:c>
-      <x:c r="B16" s="39" t="str">
+      <x:c r="B17" s="39" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="C16" s="39" t="str">
+      <x:c r="C17" s="39" t="str">
         <x:v>逐秒检查 38936 点，直连缺口 12231 点，中断 0 点</x:v>
       </x:c>
     </x:row>
@@ -8606,7 +8575,7 @@
         <x:v>3928.0643800924636</x:v>
       </x:c>
       <x:c r="K7" s="26" t="n">
-        <x:v>1.106818329020721</x:v>
+        <x:v>1.1159849956873877</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -8626,22 +8595,22 @@
         <x:v>109.2835966</x:v>
       </x:c>
       <x:c r="F8" s="18" t="n">
-        <x:v>23.0299769</x:v>
+        <x:v>23.0175933</x:v>
       </x:c>
       <x:c r="G8" s="24" t="n">
-        <x:v>716.1956176757812</x:v>
+        <x:v>726.6973876953125</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
-        <x:v>750.6049005426124</x:v>
+        <x:v>725.8760198745433</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
         <x:v>2686</x:v>
       </x:c>
       <x:c r="J8" s="24" t="n">
-        <x:v>3275.646202015594</x:v>
+        <x:v>3251.792468849153</x:v>
       </x:c>
       <x:c r="K8" s="27" t="n">
-        <x:v>0.8950848596660603</x:v>
+        <x:v>0.8952649187379393</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -8658,25 +8627,25 @@
         <x:v>4228.064380092464</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:v>109.2118354</x:v>
+        <x:v>109.2135854</x:v>
       </x:c>
       <x:c r="F9" s="18" t="n">
-        <x:v>23.01896405</x:v>
+        <x:v>23.02146405</x:v>
       </x:c>
       <x:c r="G9" s="24" t="n">
-        <x:v>586.2146301269531</x:v>
+        <x:v>538.5837554931641</x:v>
       </x:c>
       <x:c r="H9" s="24" t="n">
-        <x:v>4703.824952219404</x:v>
+        <x:v>4692.774413082056</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
         <x:v>7377</x:v>
       </x:c>
       <x:c r="J9" s="24" t="n">
-        <x:v>7680.97012463752</x:v>
+        <x:v>7665.950345947355</x:v>
       </x:c>
       <x:c r="K9" s="27" t="n">
-        <x:v>0.9541267986512145</x:v>
+        <x:v>0.9629827717764552</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -8690,7 +8659,7 @@
         <x:v>R-BAT-04</x:v>
       </x:c>
       <x:c r="D10" s="25" t="n">
-        <x:v>3575.646202015594</x:v>
+        <x:v>3551.792468849153</x:v>
       </x:c>
       <x:c r="E10" s="19" t="n">
         <x:v>109.2262272</x:v>
@@ -8702,7 +8671,7 @@
         <x:v>539.3646392822266</x:v>
       </x:c>
       <x:c r="H10" s="25" t="n">
-        <x:v>4324.243056881041</x:v>
+        <x:v>4300.3893237146</x:v>
       </x:c>
       <x:c r="I10" s="25" t="n">
         <x:v>7705</x:v>
@@ -8711,7 +8680,7 @@
         <x:v>8277.9022414723</x:v>
       </x:c>
       <x:c r="K10" s="28" t="n">
-        <x:v>1.3479619711661865</x:v>
+        <x:v>1.364417278522599</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8794,7 +8763,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
         <x:v>G01直连</x:v>
@@ -8809,10 +8778,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C8" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="D8" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -8829,7 +8798,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C9" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="D9" s="24" t="n">
         <x:v>2007.8</x:v>
@@ -8850,7 +8819,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -8865,10 +8834,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="D11" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -8885,7 +8854,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C12" s="24" t="n">
-        <x:v>1606</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="D12" s="24" t="n">
         <x:v>2007.8</x:v>
@@ -8942,7 +8911,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D15" s="24" t="n">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="E15" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -8957,10 +8926,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C16" s="24" t="n">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D16" s="24" t="n">
-        <x:v>1554</x:v>
+        <x:v>1555</x:v>
       </x:c>
       <x:c r="E16" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -8977,7 +8946,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C17" s="24" t="n">
-        <x:v>1554</x:v>
+        <x:v>1555</x:v>
       </x:c>
       <x:c r="D17" s="24" t="n">
         <x:v>1930.9</x:v>
@@ -8998,7 +8967,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D18" s="24" t="n">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="E18" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9013,10 +8982,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C19" s="24" t="n">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="D19" s="24" t="n">
-        <x:v>1146</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="E19" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -9033,7 +9002,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C20" s="24" t="n">
-        <x:v>1146</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="D20" s="24" t="n">
         <x:v>1517.5</x:v>
@@ -9054,7 +9023,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D21" s="24" t="n">
-        <x:v>850</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="E21" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9069,10 +9038,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C22" s="24" t="n">
-        <x:v>850</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="D22" s="24" t="n">
-        <x:v>1483</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="E22" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -9089,7 +9058,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C23" s="24" t="n">
-        <x:v>1483</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="D23" s="24" t="n">
         <x:v>1996</x:v>
@@ -9110,7 +9079,7 @@
         <x:v>1517.5</x:v>
       </x:c>
       <x:c r="D24" s="24" t="n">
-        <x:v>2274</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="E24" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9125,10 +9094,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C25" s="24" t="n">
-        <x:v>2274</x:v>
+        <x:v>2273</x:v>
       </x:c>
       <x:c r="D25" s="24" t="n">
-        <x:v>2686</x:v>
+        <x:v>2687</x:v>
       </x:c>
       <x:c r="E25" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -9145,7 +9114,7 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C26" s="24" t="n">
-        <x:v>2686</x:v>
+        <x:v>2687</x:v>
       </x:c>
       <x:c r="D26" s="24" t="n">
         <x:v>3072.1</x:v>
@@ -9166,7 +9135,7 @@
         <x:v>1560.9</x:v>
       </x:c>
       <x:c r="D27" s="24" t="n">
-        <x:v>2430</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="E27" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9181,10 +9150,10 @@
         <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C28" s="24" t="n">
-        <x:v>2430</x:v>
+        <x:v>2429</x:v>
       </x:c>
       <x:c r="D28" s="24" t="n">
-        <x:v>2431</x:v>
+        <x:v>2432</x:v>
       </x:c>
       <x:c r="E28" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -9201,15 +9170,17 @@
         <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C29" s="24" t="n">
-        <x:v>2431</x:v>
+        <x:v>2432</x:v>
       </x:c>
       <x:c r="D29" s="24" t="n">
-        <x:v>2433</x:v>
+        <x:v>3010</x:v>
       </x:c>
       <x:c r="E29" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F29" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str">
+        <x:v>R-M01</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="15" t="str">
@@ -9219,10 +9190,10 @@
         <x:v>阶段4</x:v>
       </x:c>
       <x:c r="C30" s="24" t="n">
-        <x:v>2433</x:v>
+        <x:v>3010</x:v>
       </x:c>
       <x:c r="D30" s="24" t="n">
-        <x:v>3009</x:v>
+        <x:v>3013</x:v>
       </x:c>
       <x:c r="E30" s="15" t="str">
         <x:v>空中中继</x:v>
@@ -9239,10 +9210,10 @@
         <x:v>阶段5</x:v>
       </x:c>
       <x:c r="C31" s="24" t="n">
-        <x:v>3009</x:v>
+        <x:v>3013</x:v>
       </x:c>
       <x:c r="D31" s="24" t="n">
-        <x:v>3011</x:v>
+        <x:v>3468.4</x:v>
       </x:c>
       <x:c r="E31" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9251,36 +9222,34 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="15" t="str">
-        <x:v>Q2-09</x:v>
+        <x:v>Q2-10</x:v>
       </x:c>
       <x:c r="B32" s="15" t="str">
-        <x:v>阶段6</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C32" s="24" t="n">
-        <x:v>3011</x:v>
+        <x:v>1693.5</x:v>
       </x:c>
       <x:c r="D32" s="24" t="n">
-        <x:v>3012</x:v>
+        <x:v>3189</x:v>
       </x:c>
       <x:c r="E32" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F32" s="15" t="str">
-        <x:v>R-M01</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F32" s="15"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="15" t="str">
-        <x:v>Q2-09</x:v>
+        <x:v>Q2-11</x:v>
       </x:c>
       <x:c r="B33" s="15" t="str">
-        <x:v>阶段7</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C33" s="24" t="n">
-        <x:v>3012</x:v>
+        <x:v>1930.9</x:v>
       </x:c>
       <x:c r="D33" s="24" t="n">
-        <x:v>3468.4</x:v>
+        <x:v>2614</x:v>
       </x:c>
       <x:c r="E33" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9289,34 +9258,36 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="15" t="str">
-        <x:v>Q2-10</x:v>
+        <x:v>Q2-11</x:v>
       </x:c>
       <x:c r="B34" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C34" s="24" t="n">
-        <x:v>1693.5</x:v>
+        <x:v>2614</x:v>
       </x:c>
       <x:c r="D34" s="24" t="n">
-        <x:v>3189</x:v>
+        <x:v>3356</x:v>
       </x:c>
       <x:c r="E34" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F34" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F34" s="15" t="str">
+        <x:v>R-M01</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="15" t="str">
         <x:v>Q2-11</x:v>
       </x:c>
       <x:c r="B35" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C35" s="24" t="n">
-        <x:v>1930.9</x:v>
+        <x:v>3356</x:v>
       </x:c>
       <x:c r="D35" s="24" t="n">
-        <x:v>2615</x:v>
+        <x:v>3690.8</x:v>
       </x:c>
       <x:c r="E35" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9325,54 +9296,54 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="15" t="str">
-        <x:v>Q2-11</x:v>
+        <x:v>Q2-12</x:v>
       </x:c>
       <x:c r="B36" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C36" s="24" t="n">
-        <x:v>2615</x:v>
+        <x:v>1996</x:v>
       </x:c>
       <x:c r="D36" s="24" t="n">
-        <x:v>3355</x:v>
+        <x:v>2745</x:v>
       </x:c>
       <x:c r="E36" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F36" s="15" t="str">
-        <x:v>R-M01</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F36" s="15"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="15" t="str">
-        <x:v>Q2-11</x:v>
+        <x:v>Q2-12</x:v>
       </x:c>
       <x:c r="B37" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C37" s="24" t="n">
-        <x:v>3355</x:v>
+        <x:v>2745</x:v>
       </x:c>
       <x:c r="D37" s="24" t="n">
-        <x:v>3690.8</x:v>
+        <x:v>3603</x:v>
       </x:c>
       <x:c r="E37" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F37" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F37" s="15" t="str">
+        <x:v>R-M01</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="15" t="str">
         <x:v>Q2-12</x:v>
       </x:c>
       <x:c r="B38" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C38" s="24" t="n">
-        <x:v>1996</x:v>
+        <x:v>3603</x:v>
       </x:c>
       <x:c r="D38" s="24" t="n">
-        <x:v>2746</x:v>
+        <x:v>4003.8</x:v>
       </x:c>
       <x:c r="E38" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9381,54 +9352,54 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="15" t="str">
-        <x:v>Q2-12</x:v>
+        <x:v>Q2-13</x:v>
       </x:c>
       <x:c r="B39" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C39" s="24" t="n">
-        <x:v>2746</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D39" s="24" t="n">
-        <x:v>3602</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="E39" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F39" s="15" t="str">
-        <x:v>R-M01</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F39" s="15"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="15" t="str">
-        <x:v>Q2-12</x:v>
+        <x:v>Q2-13</x:v>
       </x:c>
       <x:c r="B40" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C40" s="24" t="n">
-        <x:v>3602</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="D40" s="24" t="n">
-        <x:v>4003.8</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="E40" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F40" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F40" s="15" t="str">
+        <x:v>R-M02</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="15" t="str">
         <x:v>Q2-13</x:v>
       </x:c>
       <x:c r="B41" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C41" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="D41" s="24" t="n">
-        <x:v>813</x:v>
+        <x:v>1928.9623510146916</x:v>
       </x:c>
       <x:c r="E41" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9437,54 +9408,54 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="15" t="str">
-        <x:v>Q2-13</x:v>
+        <x:v>Q2-14</x:v>
       </x:c>
       <x:c r="B42" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C42" s="24" t="n">
-        <x:v>813</x:v>
+        <x:v>3362</x:v>
       </x:c>
       <x:c r="D42" s="24" t="n">
-        <x:v>1416</x:v>
+        <x:v>4324</x:v>
       </x:c>
       <x:c r="E42" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F42" s="15" t="str">
-        <x:v>R-M02</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F42" s="15"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="15" t="str">
-        <x:v>Q2-13</x:v>
+        <x:v>Q2-14</x:v>
       </x:c>
       <x:c r="B43" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C43" s="24" t="n">
-        <x:v>1416</x:v>
+        <x:v>4324</x:v>
       </x:c>
       <x:c r="D43" s="24" t="n">
-        <x:v>1928.9623510146916</x:v>
+        <x:v>5159</x:v>
       </x:c>
       <x:c r="E43" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F43" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F43" s="15" t="str">
+        <x:v>R-M04</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="15" t="str">
         <x:v>Q2-14</x:v>
       </x:c>
       <x:c r="B44" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C44" s="24" t="n">
-        <x:v>3362</x:v>
+        <x:v>5159</x:v>
       </x:c>
       <x:c r="D44" s="24" t="n">
-        <x:v>4325</x:v>
+        <x:v>5667.2</x:v>
       </x:c>
       <x:c r="E44" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9493,54 +9464,54 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="15" t="str">
-        <x:v>Q2-14</x:v>
+        <x:v>Q2-15</x:v>
       </x:c>
       <x:c r="B45" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C45" s="24" t="n">
-        <x:v>4325</x:v>
+        <x:v>3817.4</x:v>
       </x:c>
       <x:c r="D45" s="24" t="n">
-        <x:v>5158</x:v>
+        <x:v>4703</x:v>
       </x:c>
       <x:c r="E45" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F45" s="15" t="str">
-        <x:v>R-M04</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F45" s="15"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="15" t="str">
-        <x:v>Q2-14</x:v>
+        <x:v>Q2-15</x:v>
       </x:c>
       <x:c r="B46" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C46" s="24" t="n">
-        <x:v>5158</x:v>
+        <x:v>4703</x:v>
       </x:c>
       <x:c r="D46" s="24" t="n">
-        <x:v>5667.2</x:v>
+        <x:v>5709</x:v>
       </x:c>
       <x:c r="E46" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F46" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F46" s="15" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="15" t="str">
         <x:v>Q2-15</x:v>
       </x:c>
       <x:c r="B47" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C47" s="24" t="n">
-        <x:v>3817.4</x:v>
+        <x:v>5709</x:v>
       </x:c>
       <x:c r="D47" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>6187.3</x:v>
       </x:c>
       <x:c r="E47" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9549,54 +9520,54 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="15" t="str">
-        <x:v>Q2-15</x:v>
+        <x:v>Q2-16</x:v>
       </x:c>
       <x:c r="B48" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C48" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>3906.5</x:v>
       </x:c>
       <x:c r="D48" s="24" t="n">
-        <x:v>5708</x:v>
+        <x:v>4703</x:v>
       </x:c>
       <x:c r="E48" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F48" s="15" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F48" s="15"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="15" t="str">
-        <x:v>Q2-15</x:v>
+        <x:v>Q2-16</x:v>
       </x:c>
       <x:c r="B49" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C49" s="24" t="n">
-        <x:v>5708</x:v>
+        <x:v>4703</x:v>
       </x:c>
       <x:c r="D49" s="24" t="n">
-        <x:v>6187.3</x:v>
+        <x:v>5552</x:v>
       </x:c>
       <x:c r="E49" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F49" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F49" s="15" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="15" t="str">
         <x:v>Q2-16</x:v>
       </x:c>
       <x:c r="B50" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C50" s="24" t="n">
-        <x:v>3906.5</x:v>
+        <x:v>5552</x:v>
       </x:c>
       <x:c r="D50" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>5986.8</x:v>
       </x:c>
       <x:c r="E50" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9605,54 +9576,54 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="15" t="str">
-        <x:v>Q2-16</x:v>
+        <x:v>Q2-17</x:v>
       </x:c>
       <x:c r="B51" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C51" s="24" t="n">
-        <x:v>4704</x:v>
+        <x:v>4813.7</x:v>
       </x:c>
       <x:c r="D51" s="24" t="n">
-        <x:v>5551</x:v>
+        <x:v>5522</x:v>
       </x:c>
       <x:c r="E51" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F51" s="15" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F51" s="15"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="15" t="str">
-        <x:v>Q2-16</x:v>
+        <x:v>Q2-17</x:v>
       </x:c>
       <x:c r="B52" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C52" s="24" t="n">
-        <x:v>5551</x:v>
+        <x:v>5522</x:v>
       </x:c>
       <x:c r="D52" s="24" t="n">
-        <x:v>5986.8</x:v>
+        <x:v>6046</x:v>
       </x:c>
       <x:c r="E52" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F52" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F52" s="15" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="15" t="str">
         <x:v>Q2-17</x:v>
       </x:c>
       <x:c r="B53" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C53" s="24" t="n">
-        <x:v>4813.7</x:v>
+        <x:v>6046</x:v>
       </x:c>
       <x:c r="D53" s="24" t="n">
-        <x:v>5523</x:v>
+        <x:v>6374.5</x:v>
       </x:c>
       <x:c r="E53" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9661,54 +9632,54 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="15" t="str">
-        <x:v>Q2-17</x:v>
+        <x:v>Q2-18</x:v>
       </x:c>
       <x:c r="B54" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C54" s="24" t="n">
-        <x:v>5523</x:v>
+        <x:v>5667.2</x:v>
       </x:c>
       <x:c r="D54" s="24" t="n">
-        <x:v>6045</x:v>
+        <x:v>6508</x:v>
       </x:c>
       <x:c r="E54" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F54" s="15" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F54" s="15"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="15" t="str">
-        <x:v>Q2-17</x:v>
+        <x:v>Q2-18</x:v>
       </x:c>
       <x:c r="B55" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C55" s="24" t="n">
-        <x:v>6045</x:v>
+        <x:v>6508</x:v>
       </x:c>
       <x:c r="D55" s="24" t="n">
-        <x:v>6374.5</x:v>
+        <x:v>7457</x:v>
       </x:c>
       <x:c r="E55" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F55" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F55" s="15" t="str">
+        <x:v>R-M04</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="15" t="str">
         <x:v>Q2-18</x:v>
       </x:c>
       <x:c r="B56" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C56" s="24" t="n">
-        <x:v>5667.2</x:v>
+        <x:v>7457</x:v>
       </x:c>
       <x:c r="D56" s="24" t="n">
-        <x:v>6509</x:v>
+        <x:v>7871</x:v>
       </x:c>
       <x:c r="E56" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9717,54 +9688,54 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="15" t="str">
-        <x:v>Q2-18</x:v>
+        <x:v>Q2-19</x:v>
       </x:c>
       <x:c r="B57" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C57" s="24" t="n">
-        <x:v>6509</x:v>
+        <x:v>6187.3</x:v>
       </x:c>
       <x:c r="D57" s="24" t="n">
-        <x:v>7456</x:v>
+        <x:v>7010</x:v>
       </x:c>
       <x:c r="E57" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F57" s="15" t="str">
-        <x:v>R-M04</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F57" s="15"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="15" t="str">
-        <x:v>Q2-18</x:v>
+        <x:v>Q2-19</x:v>
       </x:c>
       <x:c r="B58" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C58" s="24" t="n">
-        <x:v>7456</x:v>
+        <x:v>7010</x:v>
       </x:c>
       <x:c r="D58" s="24" t="n">
-        <x:v>7871</x:v>
+        <x:v>7706</x:v>
       </x:c>
       <x:c r="E58" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F58" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F58" s="15" t="str">
+        <x:v>R-M04</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="15" t="str">
         <x:v>Q2-19</x:v>
       </x:c>
       <x:c r="B59" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C59" s="24" t="n">
-        <x:v>6187.3</x:v>
+        <x:v>7706</x:v>
       </x:c>
       <x:c r="D59" s="24" t="n">
-        <x:v>7011</x:v>
+        <x:v>8067.4</x:v>
       </x:c>
       <x:c r="E59" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9773,54 +9744,54 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="15" t="str">
-        <x:v>Q2-19</x:v>
+        <x:v>Q2-20</x:v>
       </x:c>
       <x:c r="B60" s="15" t="str">
-        <x:v>阶段2</x:v>
+        <x:v>阶段1</x:v>
       </x:c>
       <x:c r="C60" s="24" t="n">
-        <x:v>7011</x:v>
+        <x:v>5986.8</x:v>
       </x:c>
       <x:c r="D60" s="24" t="n">
-        <x:v>7705</x:v>
+        <x:v>6787</x:v>
       </x:c>
       <x:c r="E60" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F60" s="15" t="str">
-        <x:v>R-M04</x:v>
-      </x:c>
+        <x:v>G01直连</x:v>
+      </x:c>
+      <x:c r="F60" s="15"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="15" t="str">
-        <x:v>Q2-19</x:v>
+        <x:v>Q2-20</x:v>
       </x:c>
       <x:c r="B61" s="15" t="str">
-        <x:v>阶段3</x:v>
+        <x:v>阶段2</x:v>
       </x:c>
       <x:c r="C61" s="24" t="n">
-        <x:v>7705</x:v>
+        <x:v>6787</x:v>
       </x:c>
       <x:c r="D61" s="24" t="n">
-        <x:v>8067.4</x:v>
+        <x:v>7378</x:v>
       </x:c>
       <x:c r="E61" s="15" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F61" s="15"/>
+        <x:v>空中中继</x:v>
+      </x:c>
+      <x:c r="F61" s="15" t="str">
+        <x:v>R-M03</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="15" t="str">
         <x:v>Q2-20</x:v>
       </x:c>
       <x:c r="B62" s="15" t="str">
-        <x:v>阶段1</x:v>
+        <x:v>阶段3</x:v>
       </x:c>
       <x:c r="C62" s="24" t="n">
-        <x:v>5986.8</x:v>
+        <x:v>7378</x:v>
       </x:c>
       <x:c r="D62" s="24" t="n">
-        <x:v>6788</x:v>
+        <x:v>7816.4</x:v>
       </x:c>
       <x:c r="E62" s="15" t="str">
         <x:v>G01直连</x:v>
@@ -9828,60 +9799,22 @@
       <x:c r="F62" s="15"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="15" t="str">
-        <x:v>Q2-20</x:v>
-      </x:c>
-      <x:c r="B63" s="15" t="str">
-        <x:v>阶段2</x:v>
-      </x:c>
-      <x:c r="C63" s="24" t="n">
-        <x:v>6788</x:v>
-      </x:c>
-      <x:c r="D63" s="24" t="n">
-        <x:v>7377</x:v>
-      </x:c>
-      <x:c r="E63" s="15" t="str">
-        <x:v>空中中继</x:v>
-      </x:c>
-      <x:c r="F63" s="15" t="str">
-        <x:v>R-M03</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="15" t="str">
-        <x:v>Q2-20</x:v>
-      </x:c>
-      <x:c r="B64" s="15" t="str">
-        <x:v>阶段3</x:v>
-      </x:c>
-      <x:c r="C64" s="24" t="n">
-        <x:v>7377</x:v>
-      </x:c>
-      <x:c r="D64" s="24" t="n">
-        <x:v>7816.4</x:v>
-      </x:c>
-      <x:c r="E64" s="15" t="str">
+      <x:c r="A63" s="16" t="str">
+        <x:v>Q2-21</x:v>
+      </x:c>
+      <x:c r="B63" s="16" t="str">
+        <x:v>阶段1</x:v>
+      </x:c>
+      <x:c r="C63" s="25" t="n">
+        <x:v>6374.5</x:v>
+      </x:c>
+      <x:c r="D63" s="25" t="n">
+        <x:v>7561.2</x:v>
+      </x:c>
+      <x:c r="E63" s="16" t="str">
         <x:v>G01直连</x:v>
       </x:c>
-      <x:c r="F64" s="15"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="16" t="str">
-        <x:v>Q2-21</x:v>
-      </x:c>
-      <x:c r="B65" s="16" t="str">
-        <x:v>阶段1</x:v>
-      </x:c>
-      <x:c r="C65" s="25" t="n">
-        <x:v>6374.5</x:v>
-      </x:c>
-      <x:c r="D65" s="25" t="n">
-        <x:v>7561.2</x:v>
-      </x:c>
-      <x:c r="E65" s="16" t="str">
-        <x:v>G01直连</x:v>
-      </x:c>
-      <x:c r="F65" s="16"/>
+      <x:c r="F63" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>